<commit_message>
ajout des chocs externes
</commit_message>
<xml_diff>
--- a/med_shocks.xlsx
+++ b/med_shocks.xlsx
@@ -13,7 +13,775 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="288">
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
   <si>
     <t>med_Q_2</t>
   </si>
@@ -129,7 +897,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -138,13 +906,29 @@
       <diagonal/>
     </border>
     <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -202,7 +986,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>256</v>
       </c>
       <c r="B1" s="0">
         <v>-116.6265636</v>
@@ -327,7 +1111,7 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>1</v>
+        <v>257</v>
       </c>
       <c r="B2" s="0">
         <v>-116.62946099999999</v>
@@ -452,7 +1236,7 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>2</v>
+        <v>258</v>
       </c>
       <c r="B3" s="0">
         <v>-116.63425579999998</v>
@@ -577,7 +1361,7 @@
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>3</v>
+        <v>259</v>
       </c>
       <c r="B4" s="0">
         <v>-116.63882369999999</v>
@@ -702,7 +1486,7 @@
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>4</v>
+        <v>260</v>
       </c>
       <c r="B5" s="0">
         <v>-116.64488369999999</v>
@@ -827,7 +1611,7 @@
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>5</v>
+        <v>261</v>
       </c>
       <c r="B6" s="0">
         <v>-116.65981599999999</v>
@@ -952,7 +1736,7 @@
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>6</v>
+        <v>262</v>
       </c>
       <c r="B7" s="0">
         <v>-116.6905008</v>
@@ -1077,7 +1861,7 @@
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>7</v>
+        <v>263</v>
       </c>
       <c r="B8" s="0">
         <v>-116.74011229999999</v>
@@ -1202,7 +1986,7 @@
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>8</v>
+        <v>264</v>
       </c>
       <c r="B9" s="0">
         <v>-116.81824619999999</v>
@@ -1327,7 +2111,7 @@
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>9</v>
+        <v>265</v>
       </c>
       <c r="B10" s="0">
         <v>-116.94167059999999</v>
@@ -1452,7 +2236,7 @@
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>10</v>
+        <v>266</v>
       </c>
       <c r="B11" s="0">
         <v>-117.08719099999999</v>
@@ -1577,7 +2361,7 @@
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>11</v>
+        <v>267</v>
       </c>
       <c r="B12" s="0">
         <v>-117.2552001</v>
@@ -1702,7 +2486,7 @@
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>12</v>
+        <v>268</v>
       </c>
       <c r="B13" s="0">
         <v>-117.38971629999999</v>
@@ -1827,7 +2611,7 @@
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>13</v>
+        <v>269</v>
       </c>
       <c r="B14" s="0">
         <v>-117.4813461</v>
@@ -1952,7 +2736,7 @@
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>14</v>
+        <v>270</v>
       </c>
       <c r="B15" s="0">
         <v>-117.54088949999999</v>
@@ -2077,7 +2861,7 @@
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>15</v>
+        <v>271</v>
       </c>
       <c r="B16" s="0">
         <v>-117.56886899999999</v>
@@ -2202,7 +2986,7 @@
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>16</v>
+        <v>272</v>
       </c>
       <c r="B17" s="0">
         <v>-116.66050899999999</v>
@@ -2327,7 +3111,7 @@
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>17</v>
+        <v>273</v>
       </c>
       <c r="B18" s="0">
         <v>-116.66838079999999</v>
@@ -2452,7 +3236,7 @@
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>18</v>
+        <v>274</v>
       </c>
       <c r="B19" s="0">
         <v>-116.67417329999998</v>
@@ -2577,7 +3361,7 @@
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
-        <v>19</v>
+        <v>275</v>
       </c>
       <c r="B20" s="0">
         <v>-116.68315749999999</v>
@@ -2702,7 +3486,7 @@
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
-        <v>20</v>
+        <v>276</v>
       </c>
       <c r="B21" s="0">
         <v>-116.6947819</v>
@@ -2827,7 +3611,7 @@
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>21</v>
+        <v>277</v>
       </c>
       <c r="B22" s="0">
         <v>-116.7165421</v>
@@ -2952,7 +3736,7 @@
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>22</v>
+        <v>278</v>
       </c>
       <c r="B23" s="0">
         <v>-116.75656499999999</v>
@@ -3077,7 +3861,7 @@
     </row>
     <row r="24">
       <c r="A24" s="0" t="s">
-        <v>23</v>
+        <v>279</v>
       </c>
       <c r="B24" s="0">
         <v>-116.8149335</v>
@@ -3202,7 +3986,7 @@
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>24</v>
+        <v>280</v>
       </c>
       <c r="B25" s="0">
         <v>-116.8987995</v>
@@ -3327,7 +4111,7 @@
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
-        <v>25</v>
+        <v>281</v>
       </c>
       <c r="B26" s="0">
         <v>-117.0178883</v>
@@ -3452,7 +4236,7 @@
     </row>
     <row r="27">
       <c r="A27" s="0" t="s">
-        <v>26</v>
+        <v>282</v>
       </c>
       <c r="B27" s="0">
         <v>-117.16614799999999</v>
@@ -3577,7 +4361,7 @@
     </row>
     <row r="28">
       <c r="A28" s="0" t="s">
-        <v>27</v>
+        <v>283</v>
       </c>
       <c r="B28" s="0">
         <v>-117.3211757</v>
@@ -3702,7 +4486,7 @@
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>28</v>
+        <v>284</v>
       </c>
       <c r="B29" s="0">
         <v>-117.4352495</v>
@@ -3827,7 +4611,7 @@
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
-        <v>29</v>
+        <v>285</v>
       </c>
       <c r="B30" s="0">
         <v>-117.50855589999999</v>
@@ -3952,7 +4736,7 @@
     </row>
     <row r="31">
       <c r="A31" s="0" t="s">
-        <v>30</v>
+        <v>286</v>
       </c>
       <c r="B31" s="0">
         <v>-117.55515469999999</v>
@@ -4077,7 +4861,7 @@
     </row>
     <row r="32">
       <c r="A32" s="0" t="s">
-        <v>31</v>
+        <v>287</v>
       </c>
       <c r="B32" s="0">
         <v>-117.57656259999999</v>

</xml_diff>

<commit_message>
code calibration et comparaison deux calibrations
</commit_message>
<xml_diff>
--- a/med_shocks.xlsx
+++ b/med_shocks.xlsx
@@ -13,7 +13,199 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="352">
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
+  <si>
+    <t>med_Q_2</t>
+  </si>
+  <si>
+    <t>med_Q_3</t>
+  </si>
+  <si>
+    <t>med_Q_4</t>
+  </si>
+  <si>
+    <t>med_Q_5</t>
+  </si>
+  <si>
+    <t>med_Q_6</t>
+  </si>
+  <si>
+    <t>med_Q_7</t>
+  </si>
+  <si>
+    <t>med_Q_8</t>
+  </si>
+  <si>
+    <t>med_Q_9</t>
+  </si>
+  <si>
+    <t>med_Q_10</t>
+  </si>
+  <si>
+    <t>med_Q_11</t>
+  </si>
+  <si>
+    <t>med_Q_12</t>
+  </si>
+  <si>
+    <t>med_Q_13</t>
+  </si>
+  <si>
+    <t>med_Q_14</t>
+  </si>
+  <si>
+    <t>med_Q_15</t>
+  </si>
+  <si>
+    <t>med_Q_16</t>
+  </si>
+  <si>
+    <t>med_Q_17</t>
+  </si>
+  <si>
+    <t>med_NQ_2</t>
+  </si>
+  <si>
+    <t>med_NQ_3</t>
+  </si>
+  <si>
+    <t>med_NQ_4</t>
+  </si>
+  <si>
+    <t>med_NQ_5</t>
+  </si>
+  <si>
+    <t>med_NQ_6</t>
+  </si>
+  <si>
+    <t>med_NQ_7</t>
+  </si>
+  <si>
+    <t>med_NQ_8</t>
+  </si>
+  <si>
+    <t>med_NQ_9</t>
+  </si>
+  <si>
+    <t>med_NQ_10</t>
+  </si>
+  <si>
+    <t>med_NQ_11</t>
+  </si>
+  <si>
+    <t>med_NQ_12</t>
+  </si>
+  <si>
+    <t>med_NQ_13</t>
+  </si>
+  <si>
+    <t>med_NQ_14</t>
+  </si>
+  <si>
+    <t>med_NQ_15</t>
+  </si>
+  <si>
+    <t>med_NQ_16</t>
+  </si>
+  <si>
+    <t>med_NQ_17</t>
+  </si>
   <si>
     <t>med_Q_2</t>
   </si>
@@ -897,7 +1089,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -914,11 +1106,13 @@
     <border/>
     <border/>
     <border/>
+    <border/>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true"/>
@@ -929,6 +1123,8 @@
     <xf numFmtId="22" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="true"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -986,7 +1182,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="0" t="s">
-        <v>256</v>
+        <v>320</v>
       </c>
       <c r="B1" s="0">
         <v>-116.6265636</v>
@@ -1111,7 +1307,7 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>257</v>
+        <v>321</v>
       </c>
       <c r="B2" s="0">
         <v>-116.62946099999999</v>
@@ -1236,7 +1432,7 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>258</v>
+        <v>322</v>
       </c>
       <c r="B3" s="0">
         <v>-116.63425579999998</v>
@@ -1361,7 +1557,7 @@
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>259</v>
+        <v>323</v>
       </c>
       <c r="B4" s="0">
         <v>-116.63882369999999</v>
@@ -1486,7 +1682,7 @@
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>260</v>
+        <v>324</v>
       </c>
       <c r="B5" s="0">
         <v>-116.64488369999999</v>
@@ -1611,7 +1807,7 @@
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>261</v>
+        <v>325</v>
       </c>
       <c r="B6" s="0">
         <v>-116.65981599999999</v>
@@ -1736,7 +1932,7 @@
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>262</v>
+        <v>326</v>
       </c>
       <c r="B7" s="0">
         <v>-116.6905008</v>
@@ -1861,7 +2057,7 @@
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>263</v>
+        <v>327</v>
       </c>
       <c r="B8" s="0">
         <v>-116.74011229999999</v>
@@ -1986,7 +2182,7 @@
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>264</v>
+        <v>328</v>
       </c>
       <c r="B9" s="0">
         <v>-116.81824619999999</v>
@@ -2111,7 +2307,7 @@
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>265</v>
+        <v>329</v>
       </c>
       <c r="B10" s="0">
         <v>-116.94167059999999</v>
@@ -2236,7 +2432,7 @@
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>266</v>
+        <v>330</v>
       </c>
       <c r="B11" s="0">
         <v>-117.08719099999999</v>
@@ -2361,7 +2557,7 @@
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>267</v>
+        <v>331</v>
       </c>
       <c r="B12" s="0">
         <v>-117.2552001</v>
@@ -2486,7 +2682,7 @@
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>268</v>
+        <v>332</v>
       </c>
       <c r="B13" s="0">
         <v>-117.38971629999999</v>
@@ -2611,7 +2807,7 @@
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>269</v>
+        <v>333</v>
       </c>
       <c r="B14" s="0">
         <v>-117.4813461</v>
@@ -2736,7 +2932,7 @@
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>270</v>
+        <v>334</v>
       </c>
       <c r="B15" s="0">
         <v>-117.54088949999999</v>
@@ -2861,7 +3057,7 @@
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>271</v>
+        <v>335</v>
       </c>
       <c r="B16" s="0">
         <v>-117.56886899999999</v>
@@ -2986,7 +3182,7 @@
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>272</v>
+        <v>336</v>
       </c>
       <c r="B17" s="0">
         <v>-116.66050899999999</v>
@@ -3111,7 +3307,7 @@
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>273</v>
+        <v>337</v>
       </c>
       <c r="B18" s="0">
         <v>-116.66838079999999</v>
@@ -3236,7 +3432,7 @@
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>274</v>
+        <v>338</v>
       </c>
       <c r="B19" s="0">
         <v>-116.67417329999998</v>
@@ -3361,7 +3557,7 @@
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
-        <v>275</v>
+        <v>339</v>
       </c>
       <c r="B20" s="0">
         <v>-116.68315749999999</v>
@@ -3486,7 +3682,7 @@
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
-        <v>276</v>
+        <v>340</v>
       </c>
       <c r="B21" s="0">
         <v>-116.6947819</v>
@@ -3611,7 +3807,7 @@
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>277</v>
+        <v>341</v>
       </c>
       <c r="B22" s="0">
         <v>-116.7165421</v>
@@ -3736,7 +3932,7 @@
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>278</v>
+        <v>342</v>
       </c>
       <c r="B23" s="0">
         <v>-116.75656499999999</v>
@@ -3861,7 +4057,7 @@
     </row>
     <row r="24">
       <c r="A24" s="0" t="s">
-        <v>279</v>
+        <v>343</v>
       </c>
       <c r="B24" s="0">
         <v>-116.8149335</v>
@@ -3986,7 +4182,7 @@
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>280</v>
+        <v>344</v>
       </c>
       <c r="B25" s="0">
         <v>-116.8987995</v>
@@ -4111,7 +4307,7 @@
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
-        <v>281</v>
+        <v>345</v>
       </c>
       <c r="B26" s="0">
         <v>-117.0178883</v>
@@ -4236,7 +4432,7 @@
     </row>
     <row r="27">
       <c r="A27" s="0" t="s">
-        <v>282</v>
+        <v>346</v>
       </c>
       <c r="B27" s="0">
         <v>-117.16614799999999</v>
@@ -4361,7 +4557,7 @@
     </row>
     <row r="28">
       <c r="A28" s="0" t="s">
-        <v>283</v>
+        <v>347</v>
       </c>
       <c r="B28" s="0">
         <v>-117.3211757</v>
@@ -4486,7 +4682,7 @@
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>284</v>
+        <v>348</v>
       </c>
       <c r="B29" s="0">
         <v>-117.4352495</v>
@@ -4611,7 +4807,7 @@
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
-        <v>285</v>
+        <v>349</v>
       </c>
       <c r="B30" s="0">
         <v>-117.50855589999999</v>
@@ -4736,7 +4932,7 @@
     </row>
     <row r="31">
       <c r="A31" s="0" t="s">
-        <v>286</v>
+        <v>350</v>
       </c>
       <c r="B31" s="0">
         <v>-117.55515469999999</v>
@@ -4861,7 +5057,7 @@
     </row>
     <row r="32">
       <c r="A32" s="0" t="s">
-        <v>287</v>
+        <v>351</v>
       </c>
       <c r="B32" s="0">
         <v>-117.57656259999999</v>

</xml_diff>